<commit_message>
docs(crm): add Feature 2 client handover for threshold and import headers
</commit_message>
<xml_diff>
--- a/Pending-Client-Changes-Implementation-Tracker.xlsx
+++ b/Pending-Client-Changes-Implementation-Tracker.xlsx
@@ -992,7 +992,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>F2 inactive threshold default 60 days (query param 30/45/60/90). Desktop CRM only for v1. CRM list pageSize default 25 (lazy load; do not dump 3000 rows).</t>
+          <t>F2 inactive threshold + import headers — handover doc docs/Feature-2-CRM-Client-Open-Points.md (default 60d; UI 30/45/60/90; Contacts column map). Desktop CRM only v1. CRM pageSize 25 lazy load.</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>backend/seeds/clearCustomersSeed.js — do this BEFORE importing real clients.</t>
+          <t>Ran npm run seed:clear-customers — CRM already empty (0 customers). Wipe script OK before real import.</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Screenshot / count for handover.</t>
+          <t>Verified Customer.countDocuments()=0 after wipe. Safe to proceed with schema + import.</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>backend/models/Customer.js — additive only.</t>
+          <t>backend/models/Customer.js — additive only; included in toSafeObject.</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>backend/models/CustomerImportBatch.js — register in server.js model imports if required.</t>
+          <t>backend/models/CustomerImportBatch.js — registered in server.js.</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Search backend/routes for multer first.</t>
+          <t>xlsx already present. Installed multer. Added middleware/customerImportUpload.js (memory 5MB csv/xlsx) — no prior multer in live routes.</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Header map as one config object at top of file.</t>
+          <t>backend/services/customerImportService.js — CUSTOMER_IMPORT_HEADER_ALIASES + normalizeImportPhone + buildImportNotes.</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>backend/services/customerImportService.js — extras go in notes only (single unique phone).</t>
+          <t>customerImportService.importCustomers — smoke: seeds/testImportCustomersRow10.js</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>customerRoutes.js live arnav mount.</t>
+          <t>customerRoutes.js — POST /import before /:id; customerImportUpload.single(file).</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -2365,7 +2365,11 @@
           <t>Feature 2</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>customerRoutes.js — GET /import/:batchId before /:id.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -2395,7 +2399,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -2415,7 +2419,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Extra mobiles must not be dropped — always append to notes. Header-map must accept these client column names.</t>
+          <t>Locked in customerImportConstants.js + HEADER_ALIASES. File headers match; ~3007 rows / ~2999 with mobile.</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2451,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -2467,7 +2471,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Prefer live import so CustomerImportBatch audit exists. Source file: repo-root Contacts-24-Aug-02-31.xlsx.</t>
+          <t>npm run seed:client-customers — created=2813 merged=143 skipped=51 total_rows=3007; customers_now=2813. CustomerImportBatch audit exists.</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2503,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -2519,7 +2523,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>File has ~3007 rows; some blank-name/blank-mobile — expect created &lt; 3007.</t>
+          <t>Verified: DB=2813=file unique phones; 0 dups; sample 5/5 match; skipped=51. node seeds/testClientCustomersSeedVerify.js</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2555,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -2571,7 +2575,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>customerService.js or crmAlertService.js if file too large.</t>
+          <t>backend/services/crmAlertService.js — DEFAULT_INACTIVE_THRESHOLD_DAYS=60. Smoke: 2813 never-visited inactive at 60.</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2607,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -2623,7 +2627,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Must be registered BEFORE /:id if that would capture inactive.</t>
+          <t>customerRoutes.js — GET /inactive before /:id.</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2659,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -2675,7 +2679,7 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>frontend/src/api/arnav/customersApi.js</t>
+          <t>frontend/src/api/arnav/customersApi.js + arnav/index.js re-exports.</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2711,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -2727,7 +2731,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Match CrmHome / TaxList teal theme.</t>
+          <t>frontend/src/pages/crm/CrmImportCustomers.jsx — teal hero + crm-table; route in later row.</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2763,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2779,7 +2783,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Do not use dead DataTable.jsx.</t>
+          <t>frontend/src/pages/crm/CrmInactiveCustomers.jsx — crm-toolbar + crm-table; tab wire in next row.</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2815,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -2831,7 +2835,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Verify usePermission module is crm — do not guess a new module.</t>
+          <t>crm view for tab; Import uses crm edit → /crm/import (route next row).</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2867,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -2881,7 +2885,11 @@
           <t>Feature 2</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>/crm/inactive (view) + /crm/import (edit) in arnavRoutes.jsx.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2911,7 +2919,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -2931,7 +2939,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Desktop only v1 — no mobile inactive screen.</t>
+          <t>Import + inactive: module-hero, status-card, user-table, user-filter-btn thresholds; crm-import-dropzone in CrmHome.css. No mobile inactive screen.</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2971,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -2983,7 +2991,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Tech-lead request after seed-size concern. Today CrmHome listCustomers({limit:100}) would hide most of 3000 AND still be too heavy if limit were raised.</t>
+          <t>Approach locked in .cursor/rules/crm-lazy-load.mdc + IMPLEMENTATION_GUIDE §2.6a. Build starts row 25 (CUSTOMER_LIST_PAGE_SIZE). Today still listCustomers({limit:100}).</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3023,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -3035,7 +3043,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Mirrors MAX_WALLET_FAMILY_MEMBERS / REDO_WINDOW_DAYS pattern.</t>
+          <t>backend/constants/customerConstants.js — CUSTOMER_LIST_PAGE_SIZE=25, CUSTOMER_LIST_MAX_PAGE_SIZE=50, resolveCustomerListPageSize(). Wire in listCustomers next row.</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3075,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -3087,7 +3095,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>backend/services/customerService.js — current limit max 100 with no skip/total.</t>
+          <t>customerService.listCustomers — skip/limit + countDocuments; max pageSize 50 via resolveCustomerListPageSize. Controller still returns items[] until row 27 envelope.</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3127,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -3139,7 +3147,7 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>customerController listCustomersHandler + customersApi.js</t>
+          <t>listCustomersHandler returns paginated envelope; customersApi documents + maps limit→pageSize. CrmHome consumer update row 28.</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3179,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -3191,7 +3199,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>frontend/src/pages/crm/CrmHome.jsx — reuse crm-btn crm-btn--secondary.</t>
+          <t>CrmHome fetchCustomersPage — page 1 replace, Load more append; toolbar total from API; loadingMore separate from loading.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3231,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -3243,7 +3251,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Existing search box already calls loadCustomers — extend with page state.</t>
+          <t>CrmHome — 300ms debounced server search resets page 1; Clear/Enter/Search immediate; rows = API items only.</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3283,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -3295,7 +3303,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CrmHome currently passes customers into CrmWhatsAppOffers.</t>
+          <t>Inactive GET paginated {items,total,hasMore}; CrmInactiveCustomers Load more + server search; CrmWhatsAppOffers typeahead + server send recipients.</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3335,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -3347,7 +3355,7 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Do this after Seed 3000 verify count.</t>
+          <t>npm run test:crm-lazy-load — seeds/testCrmLazyLoad.js (requires seed:client-customers).</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3387,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -3399,7 +3407,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>MD 2.8</t>
+          <t>npm run test:import-csv-5row — seeds/testImportCustomersCsv5Row.js (MD 2.8).</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3439,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -3451,7 +3459,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>MD 2.8</t>
+          <t>npm run test:inactive-vs-invoice — seeds/testInactiveVsInvoice.js (MD 2.8).</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3491,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -3503,7 +3511,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Flag in handover; do not hardcode a single undeclared number.</t>
+          <t>Handover: docs/Feature-2-CRM-Client-Open-Points.md + IMPLEMENTATION_GUIDE §2.7. Constants DEFAULT_INACTIVE_THRESHOLD_DAYS + CLIENT_CONTACTS_COLUMN_MAP.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(packages): add amount_wallet schema, family linking, and client wallet seed
</commit_message>
<xml_diff>
--- a/Pending-Client-Changes-Implementation-Tracker.xlsx
+++ b/Pending-Client-Changes-Implementation-Tracker.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00 Overview'!$A$1:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 Late-Buffer'!$A$1:$J$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Customer-Import-CRM'!$A$1:$J$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Family-Wallet-Package'!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Family-Wallet-Package'!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Redo-Rework'!$A$1:$J$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3527,7 +3527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>backend/constants/packageConstants.js</t>
+          <t>Also CLIENT_WALLET_PACKAGE_TIERS (Bronze–Diamond buy/wallet_value; validity null).</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>backend/models/PackageMaster.js + toSafeObject</t>
+          <t>validity_days null = never expires for amount_wallet. packageMasterRoutes accepts wallet_value.</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>backend/models/CustomerPackage.js</t>
+          <t>expiry_date nullable for no-validity wallets; toSafeObject includes wallet + family count.</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -3866,39 +3866,39 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>precious packageRoutes.js</t>
+          <t>Live RBAC has no packages module — used billing.edit. Sale path sets wallet_balance + null expiry.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Redemption</t>
+          <t>Wallet</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Eligible wallet packages</t>
+          <t>Seed client Bronze–Diamond wallets</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>batchValidatePackageRedemptions also finds amount_wallet active not expired wallet_balance&gt;0 where customer is buyer OR in linked_family_customer_ids.</t>
+          <t>Upsert 5 amount_wallet masters from CLIENT_WALLET_PACKAGE_TIERS (no validity).</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>packageRedemptionService.js</t>
+          <t>npm run seed:client-wallet-packages</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>pricing mode wallet_deduct</t>
+          <t>Eligible wallet packages</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3945,12 +3945,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>deduction = min(lineTotal wallet_balance); remainingCharge = lineTotal - deduction. Invoice not rejected if remainingCharge &gt; 0 — remainder via cash/UPI/card.</t>
+          <t>batchValidatePackageRedemptions also finds amount_wallet active not expired wallet_balance&gt;0 where customer is buyer OR in linked_family_customer_ids.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Mirror existing full_cover/discount_pct switch in billingController.</t>
+          <t>Ownership buyer|family; getActivePackagesByCustomerId includes family wallets.</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Decrement wallet in createInvoice txn</t>
+          <t>pricing mode wallet_deduct</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -3997,12 +3997,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>findOneAndUpdate $inc wallet_balance -deduction. If hits 0 set status exhausted. Same pattern as credits_remaining.</t>
+          <t>deduction = min(lineTotal wallet_balance); remainingCharge = lineTotal - deduction. Invoice not rejected if remainingCharge &gt; 0 — remainder via cash/UPI/card.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>billingService.js withTransaction</t>
+          <t>computePackagePricing wallet_deduct + sequential allocate in billingController.</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>GST at purchase not redemption</t>
+          <t>Decrement wallet in createInvoice txn</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -4049,12 +4049,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Wallet sale taxed like package purchase. Redemption lines tax_rate 0 like prepaid_bundle. Flag default for client.</t>
+          <t>findOneAndUpdate $inc wallet_balance -deduction. If hits 0 set status exhausted. Same pattern as credits_remaining.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>resolveTax package branch — one-line if client later wants GST on redeem.</t>
+          <t>billingService.js withTransaction</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>voidInvoice restores wallet</t>
+          <t>GST at purchase not redemption</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -4101,12 +4101,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>voidInvoice reverses wallet_balance the same way it reverses credits_remaining.</t>
+          <t>Wallet sale taxed like package purchase. Redemption lines tax_rate 0 like prepaid_bundle. Flag default for client.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -4126,39 +4126,39 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Required by MD 3.7</t>
+          <t>package_covers_tax true for wallet_deduct; item_type package already 0%.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Redemption</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>PackageMasterForm third type</t>
+          <t>voidInvoice restores wallet</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Radio/select amount_wallet. Show name price wallet_value (default=price) validity_days is_active. Hide credits/included_services/discount JSON. Extend existing type switch.</t>
+          <t>voidInvoice reverses wallet_balance the same way it reverses credits_remaining.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Match PackageMasterForm teal modal/theme already used.</t>
+          <t>wallet_deduction_amount on InvoiceLineItem for restore amount.</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>PackageSale family panel</t>
+          <t>PackageMasterForm third type</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -4205,12 +4205,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>After selling amount_wallet: search existing customers (searchCustomers) + findOrCreateCustomer. List members with remove. Max 6.</t>
+          <t>Radio/select amount_wallet. Show name price wallet_value (default=price) validity_days is_active. Hide credits/included_services/discount JSON. Extend existing type switch.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Reuse POS customer picker patterns not a new design.</t>
+          <t>amount_wallet type + wallet_value; blank validity = never expires. Teal selection styles.</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>CustomerPackageList wallet display</t>
+          <t>PackageSale family panel</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Show ₹ wallet_balance not credits. Family: N chip opens same family panel.</t>
+          <t>After selling amount_wallet: search existing customers (searchCustomers) + findOrCreateCustomer. List members with remove. Max 6.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Existing list page styles.</t>
+          <t>Reuse POS customer picker patterns not a new design.</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4299,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>PosScreen wallet redeem</t>
+          <t>CustomerPackageList wallet display</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>getEligiblePackageForLine includes family wallets. Toggle shows Wallet applied -₹X remaining ₹Y. Remainder stays payable. Same POS cart chrome.</t>
+          <t>Show ₹ wallet_balance not credits. Family: N chip opens same family panel.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>PosScreen.jsx live only.</t>
+          <t>Existing list page styles.</t>
         </is>
       </c>
     </row>
@@ -4346,12 +4346,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Family + wallet API wrappers</t>
+          <t>PosScreen wallet redeem</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Thin wrappers under precious or packages API folder; re-export.</t>
+          <t>getEligiblePackageForLine includes family wallets. Toggle shows Wallet applied -₹X remaining ₹Y. Remainder stays payable. Same POS cart chrome.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -4384,7 +4384,11 @@
           <t>Feature 3</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>PosScreen.jsx live only.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -4394,12 +4398,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Routes</t>
+          <t>API</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>No dead package pages</t>
+          <t>Family + wallet API wrappers</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -4409,7 +4413,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Register only in live precious/arnav routes. Do not edit AppRoutes.jsx dead tree.</t>
+          <t>Thin wrappers under precious or packages API folder; re-export.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -4432,36 +4436,32 @@
           <t>Feature 3</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>MD 0.3</t>
-        </is>
-      </c>
+      <c r="J18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Routes</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Sell wallet + family redeem</t>
+          <t>No dead package pages</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>A buys ₹10000; add B; B ₹450 service → balance 9550; line GST 0.</t>
+          <t>Register only in live precious/arnav routes. Do not edit AppRoutes.jsx dead tree.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>MD 3.7</t>
+          <t>MD 0.3</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Overspend remainder</t>
+          <t>Sell wallet + family redeem</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Balance 200 service 500 → charge 300 via payment mode; wallet 0 exhausted.</t>
+          <t>A buys ₹10000; add B; B ₹450 service → balance 9550; line GST 0.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -4536,7 +4536,11 @@
           <t>Feature 3</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>MD 3.7</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -4551,7 +4555,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Remove family member</t>
+          <t>Overspend remainder</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -4561,7 +4565,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>B no longer eligible at POS after remove.</t>
+          <t>Balance 200 service 500 → charge 300 via payment mode; wallet 0 exhausted.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -4576,7 +4580,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -4599,7 +4603,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Void restores wallet</t>
+          <t>Remove family member</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -4609,7 +4613,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Void the ₹450 invoice → balance back to 10000.</t>
+          <t>B no longer eligible at POS after remove.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -4624,7 +4628,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -4637,57 +4641,105 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Void restores wallet</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Void the ₹450 invoice → balance back to 10000.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Arnav</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Feature 3</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t>Open points</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>GST overspend max family refund</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Coded: GST at purchase; pay difference; max 6; refund out of scope.</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Arnav</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Arnav</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Feature 3</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>MD 3.6 — flag do not build refund.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J23"/>
+  <autoFilter ref="A1:J24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>